<commit_message>
replace db_rsvoice and new python archive
</commit_message>
<xml_diff>
--- a/teste_erictel.xlsx
+++ b/teste_erictel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Serratec\mini_cruso_python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92BE2A16-9EAA-49F7-99E2-43422D5186FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0AA06ED-A4A6-4250-9D75-9F0BABE55FD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C7ED0B75-7CA6-4F1D-B827-E40683B57708}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="64">
   <si>
     <t>cod_aparelho</t>
   </si>
@@ -36,9 +36,6 @@
     <t>mac_aparelho</t>
   </si>
   <si>
-    <t>ip_aparelho</t>
-  </si>
-  <si>
     <t>data_instalação</t>
   </si>
   <si>
@@ -111,9 +108,6 @@
     <t>SECRETARIA DE OBRAS</t>
   </si>
   <si>
-    <t>COORDENACAO</t>
-  </si>
-  <si>
     <t>SIPT30</t>
   </si>
   <si>
@@ -129,10 +123,100 @@
     <t>DIOGO</t>
   </si>
   <si>
-    <t>GRP2602</t>
-  </si>
-  <si>
     <t>tipo_ip_aparelho</t>
+  </si>
+  <si>
+    <t>HT812</t>
+  </si>
+  <si>
+    <t>URA</t>
+  </si>
+  <si>
+    <t>WEBEX</t>
+  </si>
+  <si>
+    <t>T30P</t>
+  </si>
+  <si>
+    <t>T31P</t>
+  </si>
+  <si>
+    <t>GRAND_GXP1610</t>
+  </si>
+  <si>
+    <t>GRAND_GXP1615</t>
+  </si>
+  <si>
+    <t>GRAND_GRP2601</t>
+  </si>
+  <si>
+    <t>YEALINK_SIPT30</t>
+  </si>
+  <si>
+    <t>GATEWAY_HT812</t>
+  </si>
+  <si>
+    <t>PABX_URA</t>
+  </si>
+  <si>
+    <t>DIGITAL_WEBEX</t>
+  </si>
+  <si>
+    <t>YEALINK_T30P</t>
+  </si>
+  <si>
+    <t>YEALINK_T31P</t>
+  </si>
+  <si>
+    <t>EC:74:D7:64:A1:60</t>
+  </si>
+  <si>
+    <t>C0:74:AD:88:7E:BF</t>
+  </si>
+  <si>
+    <t>EC:74:D7:6D:32:78</t>
+  </si>
+  <si>
+    <t>44:DB:D2:56:1C:AD</t>
+  </si>
+  <si>
+    <t>C0:74:AD:5A:CE:8E</t>
+  </si>
+  <si>
+    <t>44:DB:D2:43:97:6A</t>
+  </si>
+  <si>
+    <t>24:9A:B8:82:8B:D3</t>
+  </si>
+  <si>
+    <t>patrimonio_aparelho</t>
+  </si>
+  <si>
+    <t>SECRETARIA DE SANEAMENTO</t>
+  </si>
+  <si>
+    <t>SECRETARIA DE DESENVOLVIMENTO SOCIAL</t>
+  </si>
+  <si>
+    <t>GARAGEM</t>
+  </si>
+  <si>
+    <t>ARQUIVO</t>
+  </si>
+  <si>
+    <t>OBRAS 1</t>
+  </si>
+  <si>
+    <t>CRAS RECEPCAO</t>
+  </si>
+  <si>
+    <t>INICIADA</t>
+  </si>
+  <si>
+    <t>PDR</t>
+  </si>
+  <si>
+    <t>PEDRO</t>
   </si>
 </sst>
 </file>
@@ -168,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -177,6 +261,15 @@
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -492,17 +585,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBD9B75F-2223-4AB7-AD06-BA8C58019F60}">
-  <dimension ref="B1:N6"/>
+  <dimension ref="B1:N20"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.25" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.75" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.625" style="6" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20.375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="38" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="15.625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.625" style="3" bestFit="1" customWidth="1"/>
@@ -510,77 +603,83 @@
     <col min="14" max="14" width="22.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
+    <row r="1" spans="2:14" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" s="7" t="s">
         <v>10</v>
-      </c>
-      <c r="N1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2">
+        <v>834</v>
+      </c>
+      <c r="E2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="G2" s="6">
+        <v>46359</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="1">
-        <v>46359</v>
-      </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" t="s">
         <v>14</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>15</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>16</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" t="s">
         <v>18</v>
-      </c>
-      <c r="M2" t="s">
-        <v>19</v>
       </c>
       <c r="N2" s="2">
         <v>20</v>
@@ -588,34 +687,40 @@
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3">
+        <v>1356</v>
+      </c>
+      <c r="E3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="6">
+        <v>46360</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" t="s">
         <v>20</v>
       </c>
-      <c r="C3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="1">
-        <v>46360</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3" t="s">
-        <v>21</v>
-      </c>
       <c r="J3" t="s">
+        <v>15</v>
+      </c>
+      <c r="K3" t="s">
         <v>16</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="M3" t="s">
         <v>18</v>
-      </c>
-      <c r="M3" t="s">
-        <v>19</v>
       </c>
       <c r="N3" s="2">
         <v>32</v>
@@ -623,34 +728,40 @@
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4">
+        <v>2410</v>
+      </c>
+      <c r="E4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="6">
+        <v>46361</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" t="s">
         <v>22</v>
       </c>
-      <c r="C4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="1">
-        <v>46361</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I4" t="s">
-        <v>21</v>
-      </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>23</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="L4" s="4" t="s">
+      <c r="M4" t="s">
         <v>25</v>
-      </c>
-      <c r="M4" t="s">
-        <v>26</v>
       </c>
       <c r="N4" s="2">
         <v>2</v>
@@ -658,73 +769,240 @@
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>27</v>
+      </c>
+      <c r="D5">
+        <v>2717</v>
+      </c>
+      <c r="E5" t="s">
+        <v>50</v>
       </c>
       <c r="F5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="6">
+        <v>46363</v>
+      </c>
+      <c r="H5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="1">
-        <v>46362</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="I5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J5" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="K5" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="M5" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="N5" s="2">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C6" t="s">
-        <v>29</v>
+        <v>33</v>
+      </c>
+      <c r="D6">
+        <v>3188</v>
+      </c>
+      <c r="E6" t="s">
+        <v>51</v>
       </c>
       <c r="F6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="6">
+        <v>46364</v>
+      </c>
+      <c r="H6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="1">
-        <v>46363</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="I6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" t="s">
+        <v>59</v>
+      </c>
+      <c r="K6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="M6" t="s">
+        <v>63</v>
+      </c>
+      <c r="N6" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="6">
+        <v>46365</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I7" t="s">
+        <v>26</v>
+      </c>
+      <c r="J7" t="s">
+        <v>58</v>
+      </c>
+      <c r="K7" t="s">
+        <v>16</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="M7" t="s">
+        <v>63</v>
+      </c>
+      <c r="N7" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="6">
+        <v>46366</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8" t="s">
+        <v>55</v>
+      </c>
+      <c r="J8" t="s">
+        <v>15</v>
+      </c>
+      <c r="K8" t="s">
+        <v>23</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="M8" t="s">
+        <v>18</v>
+      </c>
+      <c r="N8" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9">
+        <v>2807</v>
+      </c>
+      <c r="E9" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="6">
+        <v>46367</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I9" t="s">
+        <v>28</v>
+      </c>
+      <c r="J9" t="s">
+        <v>57</v>
+      </c>
+      <c r="K9" t="s">
+        <v>23</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="M9" t="s">
+        <v>25</v>
+      </c>
+      <c r="N9" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10">
+        <v>1337</v>
+      </c>
+      <c r="E10" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="6">
+        <v>46368</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I10" t="s">
+        <v>56</v>
+      </c>
+      <c r="J10" t="s">
+        <v>60</v>
+      </c>
+      <c r="K10" t="s">
+        <v>61</v>
+      </c>
+      <c r="L10" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="J6" t="s">
-        <v>16</v>
-      </c>
-      <c r="K6" t="s">
+      <c r="M10" t="s">
         <v>31</v>
       </c>
-      <c r="L6" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="M6" t="s">
-        <v>33</v>
-      </c>
-      <c r="N6" s="2">
-        <v>11</v>
-      </c>
+      <c r="N10" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I20" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
database tratament with columns
</commit_message>
<xml_diff>
--- a/teste_erictel.xlsx
+++ b/teste_erictel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Serratec\mini_cruso_python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0AA06ED-A4A6-4250-9D75-9F0BABE55FD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E49F854-2879-4C40-AC1F-E03438AA9FC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C7ED0B75-7CA6-4F1D-B827-E40683B57708}"/>
   </bookViews>
@@ -585,424 +585,424 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBD9B75F-2223-4AB7-AD06-BA8C58019F60}">
-  <dimension ref="B1:N20"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="15.25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.75" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26.625" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="38" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.625" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.25" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="22.25" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.625" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="38" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.625" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.25" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="22.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
       <c r="B1" s="7" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>54</v>
+        <v>2</v>
       </c>
       <c r="E1" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2">
+        <v>834</v>
+      </c>
+      <c r="D2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="6">
+        <v>46359</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="L2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M2" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3">
+        <v>1356</v>
+      </c>
+      <c r="D3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="6">
+        <v>46360</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="L3" t="s">
+        <v>18</v>
+      </c>
+      <c r="M3" s="2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4">
+        <v>2410</v>
+      </c>
+      <c r="D4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="6">
+        <v>46361</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" t="s">
+        <v>25</v>
+      </c>
+      <c r="M4" s="2">
         <v>2</v>
       </c>
-      <c r="F1" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="G1" s="6" t="s">
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5">
+        <v>2717</v>
+      </c>
+      <c r="D5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="6">
+        <v>46363</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="L5" t="s">
+        <v>31</v>
+      </c>
+      <c r="M5" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6">
+        <v>3188</v>
+      </c>
+      <c r="D6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="6">
+        <v>46364</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I6" t="s">
+        <v>59</v>
+      </c>
+      <c r="J6" t="s">
+        <v>16</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="L6" t="s">
+        <v>63</v>
+      </c>
+      <c r="M6" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="6">
+        <v>46365</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" t="s">
+        <v>26</v>
+      </c>
+      <c r="I7" t="s">
+        <v>58</v>
+      </c>
+      <c r="J7" t="s">
+        <v>16</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="L7" t="s">
+        <v>63</v>
+      </c>
+      <c r="M7" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="6">
+        <v>46366</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" t="s">
+        <v>55</v>
+      </c>
+      <c r="I8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J8" t="s">
+        <v>23</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="L8" t="s">
+        <v>18</v>
+      </c>
+      <c r="M8" s="2">
         <v>3</v>
       </c>
-      <c r="H1" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="I1" s="7" t="s">
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9">
+        <v>2807</v>
+      </c>
+      <c r="D9" t="s">
+        <v>52</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="6">
+        <v>46367</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I9" t="s">
+        <v>57</v>
+      </c>
+      <c r="J9" t="s">
+        <v>23</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" t="s">
+        <v>25</v>
+      </c>
+      <c r="M9" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10">
+        <v>1337</v>
+      </c>
+      <c r="D10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="6">
+        <v>46368</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" t="s">
+        <v>56</v>
+      </c>
+      <c r="I10" t="s">
+        <v>60</v>
+      </c>
+      <c r="J10" t="s">
+        <v>61</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="L10" t="s">
+        <v>31</v>
+      </c>
+      <c r="M10" s="2">
         <v>5</v>
       </c>
-      <c r="J1" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="L1" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="M1" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="N1" s="7" t="s">
-        <v>10</v>
-      </c>
     </row>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2">
-        <v>834</v>
-      </c>
-      <c r="E2" t="s">
-        <v>47</v>
-      </c>
-      <c r="F2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="6">
-        <v>46359</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J2" t="s">
-        <v>15</v>
-      </c>
-      <c r="K2" t="s">
-        <v>16</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="M2" t="s">
-        <v>18</v>
-      </c>
-      <c r="N2" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3">
-        <v>1356</v>
-      </c>
-      <c r="E3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="6">
-        <v>46360</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" t="s">
-        <v>15</v>
-      </c>
-      <c r="K3" t="s">
-        <v>16</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="M3" t="s">
-        <v>18</v>
-      </c>
-      <c r="N3" s="2">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4">
-        <v>2410</v>
-      </c>
-      <c r="E4" t="s">
-        <v>49</v>
-      </c>
-      <c r="F4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="6">
-        <v>46361</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I4" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" t="s">
-        <v>22</v>
-      </c>
-      <c r="K4" t="s">
-        <v>23</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="M4" t="s">
-        <v>25</v>
-      </c>
-      <c r="N4" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5">
-        <v>2717</v>
-      </c>
-      <c r="E5" t="s">
-        <v>50</v>
-      </c>
-      <c r="F5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="6">
-        <v>46363</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I5" t="s">
-        <v>28</v>
-      </c>
-      <c r="J5" t="s">
-        <v>15</v>
-      </c>
-      <c r="K5" t="s">
-        <v>29</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="M5" t="s">
-        <v>31</v>
-      </c>
-      <c r="N5" s="2">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6">
-        <v>3188</v>
-      </c>
-      <c r="E6" t="s">
-        <v>51</v>
-      </c>
-      <c r="F6" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="6">
-        <v>46364</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I6" t="s">
-        <v>26</v>
-      </c>
-      <c r="J6" t="s">
-        <v>59</v>
-      </c>
-      <c r="K6" t="s">
-        <v>16</v>
-      </c>
-      <c r="L6" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="M6" t="s">
-        <v>63</v>
-      </c>
-      <c r="N6" s="2">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C7" t="s">
-        <v>34</v>
-      </c>
-      <c r="F7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" s="6">
-        <v>46365</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I7" t="s">
-        <v>26</v>
-      </c>
-      <c r="J7" t="s">
-        <v>58</v>
-      </c>
-      <c r="K7" t="s">
-        <v>16</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="M7" t="s">
-        <v>63</v>
-      </c>
-      <c r="N7" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
-        <v>44</v>
-      </c>
-      <c r="C8" t="s">
-        <v>35</v>
-      </c>
-      <c r="F8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" s="6">
-        <v>46366</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I8" t="s">
-        <v>55</v>
-      </c>
-      <c r="J8" t="s">
-        <v>15</v>
-      </c>
-      <c r="K8" t="s">
-        <v>23</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="M8" t="s">
-        <v>18</v>
-      </c>
-      <c r="N8" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
-        <v>45</v>
-      </c>
-      <c r="C9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9">
-        <v>2807</v>
-      </c>
-      <c r="E9" t="s">
-        <v>52</v>
-      </c>
-      <c r="F9" t="s">
-        <v>12</v>
-      </c>
-      <c r="G9" s="6">
-        <v>46367</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J9" t="s">
-        <v>57</v>
-      </c>
-      <c r="K9" t="s">
-        <v>23</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="M9" t="s">
-        <v>25</v>
-      </c>
-      <c r="N9" s="2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
-        <v>46</v>
-      </c>
-      <c r="C10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10">
-        <v>1337</v>
-      </c>
-      <c r="E10" t="s">
-        <v>53</v>
-      </c>
-      <c r="F10" t="s">
-        <v>12</v>
-      </c>
-      <c r="G10" s="6">
-        <v>46368</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I10" t="s">
-        <v>56</v>
-      </c>
-      <c r="J10" t="s">
-        <v>60</v>
-      </c>
-      <c r="K10" t="s">
-        <v>61</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="M10" t="s">
-        <v>31</v>
-      </c>
-      <c r="N10" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="20" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I20" s="5"/>
+    <row r="20" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H20" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
acertos em funcoes de soma no main
</commit_message>
<xml_diff>
--- a/teste_erictel.xlsx
+++ b/teste_erictel.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Serratec\mini_cruso_python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E49F854-2879-4C40-AC1F-E03438AA9FC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36D51E62-3B2E-4824-9E2C-C6776A7B6154}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C7ED0B75-7CA6-4F1D-B827-E40683B57708}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="67">
   <si>
     <t>cod_aparelho</t>
   </si>
@@ -217,6 +217,15 @@
   </si>
   <si>
     <t>PEDRO</t>
+  </si>
+  <si>
+    <t>EE:DF:8A:1C:57:9C</t>
+  </si>
+  <si>
+    <t>EE:DF:65:C2:AA:1B</t>
+  </si>
+  <si>
+    <t>qtd_aparelhos_setor</t>
   </si>
 </sst>
 </file>
@@ -585,7 +594,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBD9B75F-2223-4AB7-AD06-BA8C58019F60}">
-  <dimension ref="A1:M20"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.25" bestFit="1" customWidth="1"/>
@@ -601,9 +610,10 @@
     <col min="11" max="11" width="10.625" style="3" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16.25" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="22.25" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -643,8 +653,11 @@
       <c r="M1" s="7" t="s">
         <v>10</v>
       </c>
+      <c r="N1" s="7" t="s">
+        <v>66</v>
+      </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>38</v>
       </c>
@@ -684,8 +697,12 @@
       <c r="M2" s="2">
         <v>20</v>
       </c>
+      <c r="N2" s="2">
+        <f>SUM(M3)</f>
+        <v>32</v>
+      </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>39</v>
       </c>
@@ -726,7 +743,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>40</v>
       </c>
@@ -767,7 +784,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>41</v>
       </c>
@@ -808,7 +825,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>42</v>
       </c>
@@ -849,13 +866,19 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>43</v>
       </c>
       <c r="B7" t="s">
         <v>34</v>
       </c>
+      <c r="C7" s="2">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>64</v>
+      </c>
       <c r="E7" t="s">
         <v>12</v>
       </c>
@@ -884,13 +907,19 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>44</v>
       </c>
       <c r="B8" t="s">
         <v>35</v>
       </c>
+      <c r="C8">
+        <v>10</v>
+      </c>
+      <c r="D8" t="s">
+        <v>65</v>
+      </c>
       <c r="E8" t="s">
         <v>12</v>
       </c>
@@ -919,7 +948,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>45</v>
       </c>
@@ -960,7 +989,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>46</v>
       </c>

</xml_diff>